<commit_message>
Battery mass parameter updated
</commit_message>
<xml_diff>
--- a/Parameter Exchange.xlsx
+++ b/Parameter Exchange.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2705" uniqueCount="430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2706" uniqueCount="431">
   <si>
     <t>CSS</t>
   </si>
@@ -1440,6 +1440,9 @@
   </si>
   <si>
     <t>0.7227829891521151</t>
+  </si>
+  <si>
+    <t>69.9442520917341</t>
   </si>
 </sst>
 </file>
@@ -1458,7 +1461,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="0"/>
+      <color theme="0" rgb="FFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1917,8 +1920,8 @@
   <dimension ref="A1:J141"/>
   <sheetFormatPr defaultColWidth="21.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.28515625" customWidth="true"/>
-    <col min="5" max="5" width="59.140625" customWidth="true"/>
+    <col min="1" max="1" customWidth="true" width="40.28515625"/>
+    <col min="5" max="5" customWidth="true" width="59.140625"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="true" x14ac:dyDescent="0.25">
@@ -1978,7 +1981,7 @@
       <c r="G3" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H3"/>
+      <c r="H3" s="0"/>
     </row>
     <row r="4" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
@@ -2002,7 +2005,7 @@
       <c r="G4" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H4"/>
+      <c r="H4" s="0"/>
     </row>
     <row r="5" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
@@ -2018,7 +2021,7 @@
         <v>223</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>232</v>
@@ -2049,7 +2052,7 @@
       <c r="G6" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H6"/>
+      <c r="H6" s="0"/>
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
     </row>
@@ -2102,7 +2105,7 @@
       <c r="G8" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H8"/>
+      <c r="H8" s="0"/>
     </row>
     <row r="9" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
@@ -2178,7 +2181,7 @@
       <c r="G11" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H11"/>
+      <c r="H11" s="0"/>
     </row>
     <row r="12" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
@@ -2225,7 +2228,7 @@
       <c r="G13" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H13"/>
+      <c r="H13" s="0"/>
     </row>
     <row r="14" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
@@ -2249,7 +2252,7 @@
       <c r="G14" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H14"/>
+      <c r="H14" s="0"/>
     </row>
     <row r="15" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
@@ -2299,7 +2302,7 @@
       <c r="G16" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H16"/>
+      <c r="H16" s="0"/>
     </row>
     <row r="17" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
@@ -2323,7 +2326,7 @@
       <c r="G17" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H17"/>
+      <c r="H17" s="0"/>
     </row>
     <row r="18" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
@@ -2347,7 +2350,7 @@
       <c r="G18" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H18"/>
+      <c r="H18" s="0"/>
     </row>
     <row r="19" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
@@ -2397,7 +2400,7 @@
       <c r="G20" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H20"/>
+      <c r="H20" s="0"/>
     </row>
     <row r="21" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
@@ -2473,7 +2476,7 @@
       <c r="G23" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H23"/>
+      <c r="H23" s="0"/>
     </row>
     <row r="24" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
@@ -2523,7 +2526,7 @@
       <c r="G25" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H25"/>
+      <c r="H25" s="0"/>
     </row>
     <row r="26" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
@@ -2547,7 +2550,7 @@
       <c r="G26" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H26"/>
+      <c r="H26" s="0"/>
     </row>
     <row r="27" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
@@ -2701,7 +2704,7 @@
       <c r="G32" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H32"/>
+      <c r="H32" s="0"/>
     </row>
     <row r="33" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
@@ -2725,7 +2728,7 @@
       <c r="G33" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H33"/>
+      <c r="H33" s="0"/>
     </row>
     <row r="34" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
@@ -2749,7 +2752,7 @@
       <c r="G34" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H34"/>
+      <c r="H34" s="0"/>
     </row>
     <row r="35" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
@@ -2799,7 +2802,7 @@
       <c r="G36" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H36"/>
+      <c r="H36" s="0"/>
     </row>
     <row r="37" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
@@ -2901,7 +2904,7 @@
       <c r="G40" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H40"/>
+      <c r="H40" s="0"/>
     </row>
     <row r="41" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
@@ -2925,7 +2928,7 @@
       <c r="G41" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H41"/>
+      <c r="H41" s="0"/>
     </row>
     <row r="42" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A42" s="7" t="s">
@@ -3079,7 +3082,7 @@
       <c r="G47" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H47"/>
+      <c r="H47" s="0"/>
     </row>
     <row r="48" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
@@ -3103,7 +3106,7 @@
       <c r="G48" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H48"/>
+      <c r="H48" s="0"/>
     </row>
     <row r="49" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
@@ -3231,7 +3234,7 @@
       <c r="G53" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H53"/>
+      <c r="H53" s="0"/>
     </row>
     <row r="54" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A54" s="7" t="s">
@@ -3255,7 +3258,7 @@
       <c r="G54" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H54"/>
+      <c r="H54" s="0"/>
     </row>
     <row r="55" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
@@ -3305,7 +3308,7 @@
       <c r="G56" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H56"/>
+      <c r="H56" s="0"/>
     </row>
     <row r="57" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
@@ -3329,7 +3332,7 @@
       <c r="G57" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H57"/>
+      <c r="H57" s="0"/>
     </row>
     <row r="58" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A58" s="7" t="s">
@@ -3431,7 +3434,7 @@
       <c r="G61" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H61"/>
+      <c r="H61" s="0"/>
     </row>
     <row r="62" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
@@ -3507,7 +3510,7 @@
       <c r="G64" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H64"/>
+      <c r="H64" s="0"/>
     </row>
     <row r="65" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
@@ -3557,7 +3560,7 @@
       <c r="G66" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H66"/>
+      <c r="H66" s="0"/>
     </row>
     <row r="67" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
@@ -3581,7 +3584,7 @@
       <c r="G67" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H67"/>
+      <c r="H67" s="0"/>
     </row>
     <row r="68" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
@@ -3605,7 +3608,7 @@
       <c r="G68" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H68"/>
+      <c r="H68" s="0"/>
     </row>
     <row r="69" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
@@ -3655,7 +3658,7 @@
       <c r="G70" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H70"/>
+      <c r="H70" s="0"/>
     </row>
     <row r="71" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
@@ -4541,8 +4544,8 @@
       <c r="D106" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="E106" s="7">
-        <v>69.9442520917341</v>
+      <c r="E106" s="7" t="s">
+        <v>430</v>
       </c>
       <c r="F106" s="7" t="s">
         <v>232</v>

</xml_diff>

<commit_message>
Re-run range parametric model
</commit_message>
<xml_diff>
--- a/Parameter Exchange.xlsx
+++ b/Parameter Exchange.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
-  <workbookPr filterPrivacy="1" autoCompressPictures="0" defaultThemeVersion="124226"/>
+  <workbookPr filterPrivacy="true" autoCompressPictures="false" defaultThemeVersion="124226"/>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F56D107C-7721-4D1C-8C52-40C16289E77C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500"/>
   </bookViews>
   <sheets>
     <sheet name="Report" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Report!$A$2:$H$141</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Report!$A$2:$H$141</definedName>
   </definedNames>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029" fullCalcOnLoad="true" concurrentCalc="false"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="945" uniqueCount="417">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="945" uniqueCount="417">
   <si>
     <t>CSS</t>
   </si>
@@ -1343,8 +1343,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1396,12 +1396,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.49995422223578601"/>
+        <fgColor theme="0" tint="-0.49995422223579"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -1411,16 +1411,16 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color auto="true"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color auto="true"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color auto="true"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color auto="true"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1429,39 +1429,41 @@
       <right/>
       <top/>
       <bottom style="thin">
-        <color auto="1"/>
+        <color auto="true"/>
       </bottom>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
+      <alignment vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{E23A8A3D-9EA7-4417-AD7C-D941388C039B}"/>
+    <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -1477,7 +1479,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
     <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
@@ -1594,7 +1596,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1615,9 +1617,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin ang="16200000" scaled="true"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1638,7 +1640,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin ang="16200000" scaled="false"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -1667,7 +1669,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="false">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -1676,7 +1678,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="false">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1685,7 +1687,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="false">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1708,7 +1710,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1734,7 +1736,7 @@
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1762,15 +1764,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J141"/>
-  <sheetFormatPr defaultColWidth="21.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultColWidth="21.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="40.26953125" customWidth="1"/>
-    <col min="5" max="5" width="59.1796875" customWidth="1"/>
+    <col min="1" max="1" width="40.26953125" customWidth="true"/>
+    <col min="5" max="5" width="55.90625" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" ht="30" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1782,7 +1784,7 @@
       <c r="G1" s="6"/>
       <c r="H1" s="3"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>409</v>
       </c>
@@ -1805,7 +1807,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="3" spans="1:10" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -1829,7 +1831,7 @@
       </c>
       <c r="H3"/>
     </row>
-    <row r="4" spans="1:10" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
@@ -1853,7 +1855,7 @@
       </c>
       <c r="H4"/>
     </row>
-    <row r="5" spans="1:10" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
@@ -1876,7 +1878,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="6" spans="1:10" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
@@ -1902,7 +1904,7 @@
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
     </row>
-    <row r="7" spans="1:10" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>15</v>
       </c>
@@ -1929,7 +1931,7 @@
       </c>
       <c r="J7" s="5"/>
     </row>
-    <row r="8" spans="1:10" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>17</v>
       </c>
@@ -1953,7 +1955,7 @@
       </c>
       <c r="H8"/>
     </row>
-    <row r="9" spans="1:10" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>234</v>
       </c>
@@ -1979,7 +1981,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="10" spans="1:10" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>306</v>
       </c>
@@ -2005,7 +2007,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="11" spans="1:10" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>373</v>
       </c>
@@ -2029,7 +2031,7 @@
       </c>
       <c r="H11"/>
     </row>
-    <row r="12" spans="1:10" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>22</v>
       </c>
@@ -2052,7 +2054,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="13" spans="1:10" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>25</v>
       </c>
@@ -2076,7 +2078,7 @@
       </c>
       <c r="H13"/>
     </row>
-    <row r="14" spans="1:10" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>29</v>
       </c>
@@ -2100,7 +2102,7 @@
       </c>
       <c r="H14"/>
     </row>
-    <row r="15" spans="1:10" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>32</v>
       </c>
@@ -2126,7 +2128,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="16" spans="1:10" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>308</v>
       </c>
@@ -2150,7 +2152,7 @@
       </c>
       <c r="H16"/>
     </row>
-    <row r="17" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>310</v>
       </c>
@@ -2174,7 +2176,7 @@
       </c>
       <c r="H17"/>
     </row>
-    <row r="18" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>375</v>
       </c>
@@ -2198,7 +2200,7 @@
       </c>
       <c r="H18"/>
     </row>
-    <row r="19" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>36</v>
       </c>
@@ -2224,7 +2226,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="20" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>39</v>
       </c>
@@ -2248,7 +2250,7 @@
       </c>
       <c r="H20"/>
     </row>
-    <row r="21" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>42</v>
       </c>
@@ -2274,7 +2276,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>45</v>
       </c>
@@ -2300,7 +2302,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="23" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>377</v>
       </c>
@@ -2324,7 +2326,7 @@
       </c>
       <c r="H23"/>
     </row>
-    <row r="24" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>50</v>
       </c>
@@ -2350,7 +2352,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="25" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="25" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>53</v>
       </c>
@@ -2374,7 +2376,7 @@
       </c>
       <c r="H25"/>
     </row>
-    <row r="26" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="26" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>237</v>
       </c>
@@ -2398,7 +2400,7 @@
       </c>
       <c r="H26"/>
     </row>
-    <row r="27" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="27" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>312</v>
       </c>
@@ -2424,7 +2426,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="28" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="28" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>379</v>
       </c>
@@ -2450,7 +2452,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="29" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="29" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>56</v>
       </c>
@@ -2476,7 +2478,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="30" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>59</v>
       </c>
@@ -2502,7 +2504,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="31" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="31" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>63</v>
       </c>
@@ -2528,7 +2530,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="32" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="32" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>66</v>
       </c>
@@ -2552,7 +2554,7 @@
       </c>
       <c r="H32"/>
     </row>
-    <row r="33" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="33" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>359</v>
       </c>
@@ -2576,7 +2578,7 @@
       </c>
       <c r="H33"/>
     </row>
-    <row r="34" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="34" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>360</v>
       </c>
@@ -2600,7 +2602,7 @@
       </c>
       <c r="H34"/>
     </row>
-    <row r="35" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="35" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>380</v>
       </c>
@@ -2626,7 +2628,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="36" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="36" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>70</v>
       </c>
@@ -2650,7 +2652,7 @@
       </c>
       <c r="H36"/>
     </row>
-    <row r="37" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="37" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>73</v>
       </c>
@@ -2676,7 +2678,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="38" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="38" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>239</v>
       </c>
@@ -2702,7 +2704,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="39" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="39" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>317</v>
       </c>
@@ -2728,7 +2730,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="40" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="40" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>382</v>
       </c>
@@ -2752,7 +2754,7 @@
       </c>
       <c r="H40"/>
     </row>
-    <row r="41" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="41" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>77</v>
       </c>
@@ -2776,7 +2778,7 @@
       </c>
       <c r="H41"/>
     </row>
-    <row r="42" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="42" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>80</v>
       </c>
@@ -2802,7 +2804,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="43" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="43" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>240</v>
       </c>
@@ -2828,7 +2830,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="44" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="44" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>242</v>
       </c>
@@ -2854,7 +2856,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="45" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="45" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>244</v>
       </c>
@@ -2880,7 +2882,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="46" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="46" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>246</v>
       </c>
@@ -2906,7 +2908,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="47" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="47" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>248</v>
       </c>
@@ -2930,7 +2932,7 @@
       </c>
       <c r="H47"/>
     </row>
-    <row r="48" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="48" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>320</v>
       </c>
@@ -2954,7 +2956,7 @@
       </c>
       <c r="H48"/>
     </row>
-    <row r="49" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="49" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>322</v>
       </c>
@@ -2980,7 +2982,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="50" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="50" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>383</v>
       </c>
@@ -3006,7 +3008,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="51" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="51" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
         <v>84</v>
       </c>
@@ -3032,7 +3034,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="52" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="52" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>87</v>
       </c>
@@ -3058,7 +3060,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="53" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="53" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>250</v>
       </c>
@@ -3082,7 +3084,7 @@
       </c>
       <c r="H53"/>
     </row>
-    <row r="54" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="54" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>325</v>
       </c>
@@ -3106,7 +3108,7 @@
       </c>
       <c r="H54"/>
     </row>
-    <row r="55" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="55" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>385</v>
       </c>
@@ -3132,7 +3134,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="56" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="56" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>91</v>
       </c>
@@ -3156,7 +3158,7 @@
       </c>
       <c r="H56"/>
     </row>
-    <row r="57" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="57" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>94</v>
       </c>
@@ -3180,7 +3182,7 @@
       </c>
       <c r="H57"/>
     </row>
-    <row r="58" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="58" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>97</v>
       </c>
@@ -3206,7 +3208,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="59" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="59" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>100</v>
       </c>
@@ -3232,7 +3234,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="60" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="60" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>251</v>
       </c>
@@ -3258,7 +3260,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="61" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="61" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
         <v>253</v>
       </c>
@@ -3282,7 +3284,7 @@
       </c>
       <c r="H61"/>
     </row>
-    <row r="62" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="62" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>386</v>
       </c>
@@ -3308,7 +3310,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="63" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="63" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
         <v>105</v>
       </c>
@@ -3334,7 +3336,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="64" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="64" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
         <v>109</v>
       </c>
@@ -3358,7 +3360,7 @@
       </c>
       <c r="H64"/>
     </row>
-    <row r="65" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="65" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
         <v>112</v>
       </c>
@@ -3384,7 +3386,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="66" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="66" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
         <v>328</v>
       </c>
@@ -3408,7 +3410,7 @@
       </c>
       <c r="H66"/>
     </row>
-    <row r="67" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="67" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
         <v>330</v>
       </c>
@@ -3432,7 +3434,7 @@
       </c>
       <c r="H67"/>
     </row>
-    <row r="68" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="68" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>367</v>
       </c>
@@ -3456,7 +3458,7 @@
       </c>
       <c r="H68"/>
     </row>
-    <row r="69" spans="1:8" s="1" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="69" s="1" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>388</v>
       </c>
@@ -3482,7 +3484,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="70" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="70" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>369</v>
       </c>
@@ -3506,7 +3508,7 @@
       </c>
       <c r="H70"/>
     </row>
-    <row r="71" spans="1:8" s="5" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="71" s="5" customFormat="true" ht="14.25" customHeight="true" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
         <v>371</v>
       </c>
@@ -3532,7 +3534,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="72" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="72" ht="29" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
         <v>254</v>
       </c>
@@ -3555,7 +3557,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="73" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="73" ht="29" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
         <v>256</v>
       </c>
@@ -3581,7 +3583,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="74" ht="29" x14ac:dyDescent="0.35">
       <c r="A74" s="2" t="s">
         <v>259</v>
       </c>
@@ -3607,7 +3609,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="75" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="75" ht="29" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
         <v>261</v>
       </c>
@@ -3633,7 +3635,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="76" ht="29" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
         <v>263</v>
       </c>
@@ -3659,7 +3661,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="77" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="77" ht="29" x14ac:dyDescent="0.35">
       <c r="A77" s="2" t="s">
         <v>265</v>
       </c>
@@ -3682,7 +3684,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="78" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="78" ht="29" x14ac:dyDescent="0.35">
       <c r="A78" s="2" t="s">
         <v>267</v>
       </c>
@@ -3705,7 +3707,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="79" ht="29" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
         <v>116</v>
       </c>
@@ -3731,7 +3733,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="80" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="80" ht="29" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
         <v>119</v>
       </c>
@@ -3757,7 +3759,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="81" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="81" ht="29" x14ac:dyDescent="0.35">
       <c r="A81" s="2" t="s">
         <v>122</v>
       </c>
@@ -3783,7 +3785,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="82" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="82" ht="29" x14ac:dyDescent="0.35">
       <c r="A82" s="2" t="s">
         <v>125</v>
       </c>
@@ -3809,7 +3811,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="83" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="83" ht="29" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
         <v>390</v>
       </c>
@@ -3835,7 +3837,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="84" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="84" ht="29" x14ac:dyDescent="0.35">
       <c r="A84" s="2" t="s">
         <v>130</v>
       </c>
@@ -3858,7 +3860,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="85" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="85" ht="29" x14ac:dyDescent="0.35">
       <c r="A85" s="2" t="s">
         <v>133</v>
       </c>
@@ -3881,7 +3883,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="86" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="86" ht="29" x14ac:dyDescent="0.35">
       <c r="A86" s="2" t="s">
         <v>136</v>
       </c>
@@ -3907,7 +3909,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="87" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="87" ht="29" x14ac:dyDescent="0.35">
       <c r="A87" s="2" t="s">
         <v>141</v>
       </c>
@@ -3933,7 +3935,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="88" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="88" ht="29" x14ac:dyDescent="0.35">
       <c r="A88" s="2" t="s">
         <v>144</v>
       </c>
@@ -3959,7 +3961,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="89" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="89" ht="29" x14ac:dyDescent="0.35">
       <c r="A89" s="2" t="s">
         <v>147</v>
       </c>
@@ -3985,7 +3987,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="90" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="90" ht="29" x14ac:dyDescent="0.35">
       <c r="A90" s="2" t="s">
         <v>149</v>
       </c>
@@ -4011,7 +4013,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="91" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="91" ht="29" x14ac:dyDescent="0.35">
       <c r="A91" s="2" t="s">
         <v>392</v>
       </c>
@@ -4034,7 +4036,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="92" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="92" ht="29" x14ac:dyDescent="0.35">
       <c r="A92" s="2" t="s">
         <v>153</v>
       </c>
@@ -4057,7 +4059,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="93" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="93" ht="29" x14ac:dyDescent="0.35">
       <c r="A93" s="2" t="s">
         <v>156</v>
       </c>
@@ -4080,7 +4082,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="94" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="94" ht="29" x14ac:dyDescent="0.35">
       <c r="A94" s="2" t="s">
         <v>159</v>
       </c>
@@ -4103,7 +4105,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="95" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="95" ht="29" x14ac:dyDescent="0.35">
       <c r="A95" s="2" t="s">
         <v>162</v>
       </c>
@@ -4126,7 +4128,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="96" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="96" ht="29" x14ac:dyDescent="0.35">
       <c r="A96" s="2" t="s">
         <v>394</v>
       </c>
@@ -4149,7 +4151,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="97" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="97" ht="29" x14ac:dyDescent="0.35">
       <c r="A97" s="2" t="s">
         <v>166</v>
       </c>
@@ -4172,7 +4174,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="98" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="98" ht="29" x14ac:dyDescent="0.35">
       <c r="A98" s="2" t="s">
         <v>168</v>
       </c>
@@ -4195,7 +4197,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="99" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="99" ht="29" x14ac:dyDescent="0.35">
       <c r="A99" s="2" t="s">
         <v>171</v>
       </c>
@@ -4221,7 +4223,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="100" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="100" ht="29" x14ac:dyDescent="0.35">
       <c r="A100" s="2" t="s">
         <v>174</v>
       </c>
@@ -4247,7 +4249,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="101" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="101" ht="29" x14ac:dyDescent="0.35">
       <c r="A101" s="2" t="s">
         <v>177</v>
       </c>
@@ -4273,7 +4275,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="102" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="102" ht="29" x14ac:dyDescent="0.35">
       <c r="A102" s="2" t="s">
         <v>180</v>
       </c>
@@ -4299,7 +4301,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="103" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="103" ht="29" x14ac:dyDescent="0.35">
       <c r="A103" s="2" t="s">
         <v>183</v>
       </c>
@@ -4325,7 +4327,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="104" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="104" ht="29" x14ac:dyDescent="0.35">
       <c r="A104" s="2" t="s">
         <v>186</v>
       </c>
@@ -4351,7 +4353,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="105" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="105" ht="29" x14ac:dyDescent="0.35">
       <c r="A105" s="2" t="s">
         <v>396</v>
       </c>
@@ -4377,7 +4379,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="106" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="106" ht="29" x14ac:dyDescent="0.35">
       <c r="A106" s="2" t="s">
         <v>190</v>
       </c>
@@ -4390,8 +4392,8 @@
       <c r="D106" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="E106" s="2" t="s">
-        <v>416</v>
+      <c r="E106" s="2">
+        <v>73.014975354298031</v>
       </c>
       <c r="F106" s="2" t="s">
         <v>232</v>
@@ -4403,7 +4405,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="107" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="107" ht="29" x14ac:dyDescent="0.35">
       <c r="A107" s="2" t="s">
         <v>193</v>
       </c>
@@ -4429,7 +4431,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="108" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="108" ht="29" x14ac:dyDescent="0.35">
       <c r="A108" s="2" t="s">
         <v>195</v>
       </c>
@@ -4455,7 +4457,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="109" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="109" ht="29" x14ac:dyDescent="0.35">
       <c r="A109" s="2" t="s">
         <v>398</v>
       </c>
@@ -4478,7 +4480,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="110" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="110" ht="29" x14ac:dyDescent="0.35">
       <c r="A110" s="2" t="s">
         <v>274</v>
       </c>
@@ -4501,7 +4503,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="111" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="111" ht="29" x14ac:dyDescent="0.35">
       <c r="A111" s="2" t="s">
         <v>276</v>
       </c>
@@ -4527,7 +4529,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="112" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="112" ht="29" x14ac:dyDescent="0.35">
       <c r="A112" s="2" t="s">
         <v>278</v>
       </c>
@@ -4553,7 +4555,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="113" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="113" ht="29" x14ac:dyDescent="0.35">
       <c r="A113" s="2" t="s">
         <v>280</v>
       </c>
@@ -4579,7 +4581,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="114" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="114" ht="29" x14ac:dyDescent="0.35">
       <c r="A114" s="2" t="s">
         <v>282</v>
       </c>
@@ -4605,7 +4607,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="115" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="115" ht="29" x14ac:dyDescent="0.35">
       <c r="A115" s="2" t="s">
         <v>199</v>
       </c>
@@ -4631,7 +4633,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="116" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="116" ht="29" x14ac:dyDescent="0.35">
       <c r="A116" s="2" t="s">
         <v>202</v>
       </c>
@@ -4657,7 +4659,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="117" x14ac:dyDescent="0.35">
       <c r="A117" s="2" t="s">
         <v>333</v>
       </c>
@@ -4683,7 +4685,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="118" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="118" ht="29" x14ac:dyDescent="0.35">
       <c r="A118" s="2" t="s">
         <v>335</v>
       </c>
@@ -4709,7 +4711,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="119" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="119" ht="29" x14ac:dyDescent="0.35">
       <c r="A119" s="2" t="s">
         <v>400</v>
       </c>
@@ -4732,7 +4734,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="120" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="120" ht="29" x14ac:dyDescent="0.35">
       <c r="A120" s="2" t="s">
         <v>206</v>
       </c>
@@ -4755,7 +4757,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="121" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="121" ht="29" x14ac:dyDescent="0.35">
       <c r="A121" s="2" t="s">
         <v>209</v>
       </c>
@@ -4778,7 +4780,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="122" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="122" ht="29" x14ac:dyDescent="0.35">
       <c r="A122" s="2" t="s">
         <v>213</v>
       </c>
@@ -4801,7 +4803,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="123" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="123" ht="29" x14ac:dyDescent="0.35">
       <c r="A123" s="2" t="s">
         <v>285</v>
       </c>
@@ -4824,7 +4826,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="124" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="124" ht="29" x14ac:dyDescent="0.35">
       <c r="A124" s="2" t="s">
         <v>286</v>
       </c>
@@ -4847,7 +4849,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="125" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="125" ht="29" x14ac:dyDescent="0.35">
       <c r="A125" s="2" t="s">
         <v>288</v>
       </c>
@@ -4870,7 +4872,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="126" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="126" ht="29" x14ac:dyDescent="0.35">
       <c r="A126" s="2" t="s">
         <v>290</v>
       </c>
@@ -4893,7 +4895,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="127" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="127" ht="29" x14ac:dyDescent="0.35">
       <c r="A127" s="2" t="s">
         <v>292</v>
       </c>
@@ -4916,7 +4918,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="128" spans="1:8" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="128" ht="29" x14ac:dyDescent="0.35">
       <c r="A128" s="2" t="s">
         <v>294</v>
       </c>
@@ -4939,7 +4941,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="129" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="129" ht="29" x14ac:dyDescent="0.35">
       <c r="A129" s="2" t="s">
         <v>296</v>
       </c>
@@ -4962,7 +4964,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="130" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="130" ht="29" x14ac:dyDescent="0.35">
       <c r="A130" s="2" t="s">
         <v>298</v>
       </c>
@@ -4985,7 +4987,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="131" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="131" ht="29" x14ac:dyDescent="0.35">
       <c r="A131" s="2" t="s">
         <v>300</v>
       </c>
@@ -5008,7 +5010,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="132" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="132" ht="29" x14ac:dyDescent="0.35">
       <c r="A132" s="2" t="s">
         <v>302</v>
       </c>
@@ -5031,7 +5033,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="133" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="133" ht="29" x14ac:dyDescent="0.35">
       <c r="A133" s="2" t="s">
         <v>304</v>
       </c>
@@ -5054,7 +5056,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="134" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="134" ht="29" x14ac:dyDescent="0.35">
       <c r="A134" s="2" t="s">
         <v>338</v>
       </c>
@@ -5077,7 +5079,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="135" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="135" ht="29" x14ac:dyDescent="0.35">
       <c r="A135" s="2" t="s">
         <v>340</v>
       </c>
@@ -5100,7 +5102,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="136" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="136" ht="29" x14ac:dyDescent="0.35">
       <c r="A136" s="2" t="s">
         <v>402</v>
       </c>
@@ -5123,7 +5125,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="137" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="137" ht="29" x14ac:dyDescent="0.35">
       <c r="A137" s="2" t="s">
         <v>217</v>
       </c>
@@ -5146,7 +5148,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="138" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="138" ht="29" x14ac:dyDescent="0.35">
       <c r="A138" s="2" t="s">
         <v>221</v>
       </c>
@@ -5169,7 +5171,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="139" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="139" ht="29" x14ac:dyDescent="0.35">
       <c r="A139" s="2" t="s">
         <v>225</v>
       </c>
@@ -5192,7 +5194,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="140" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="140" ht="29" x14ac:dyDescent="0.35">
       <c r="A140" s="2" t="s">
         <v>228</v>
       </c>
@@ -5215,7 +5217,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="141" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="141" ht="29" x14ac:dyDescent="0.35">
       <c r="A141" s="2" t="s">
         <v>404</v>
       </c>
@@ -5239,7 +5241,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:H141" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A2:H141"/>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>

</xml_diff>